<commit_message>
Updated data articles raw data and data dictionary; Minor fixes to figures caps. Rendered index.
</commit_message>
<xml_diff>
--- a/data/raw/data_articles/datajournal_articles git V final_2.xlsx
+++ b/data/raw/data_articles/datajournal_articles git V final_2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bliv10\Desktop\DCC github\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C748025C-8447-4308-9ABB-9FC8B3A855E8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C748025C-8447-4308-9ABB-9FC8B3A855E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,6 +20,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -30,238 +41,238 @@
     <t>Number</t>
   </si>
   <si>
+    <t>Charité article DOI</t>
+  </si>
+  <si>
+    <t>data in repository (1 = yes, 0 = no)</t>
+  </si>
+  <si>
+    <t>dataset DOI, accession code, or link</t>
+  </si>
+  <si>
+    <t>dataset publication year (earliest version)</t>
+  </si>
+  <si>
+    <t>dataset publication year (version listed here)</t>
+  </si>
+  <si>
+    <t>license</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2016.02.047</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2016.06.021</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2016.07.009</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2016.09.012</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2017.08.034</t>
+  </si>
+  <si>
+    <t>10.1016/j.dib.2017.11.062</t>
+  </si>
+  <si>
     <t>10.1038/s41597-019-0129-z</t>
   </si>
   <si>
+    <t>https://doi.org/10.18112/openneuro.ds001875.v1.0.3</t>
+  </si>
+  <si>
+    <t>CC0</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5281/zenodo.1471588</t>
+  </si>
+  <si>
+    <t>CC-BY</t>
+  </si>
+  <si>
     <t>10.1038/s41597-019-0161-z</t>
   </si>
   <si>
+    <t>SRP136594</t>
+  </si>
+  <si>
+    <t>no versioning</t>
+  </si>
+  <si>
+    <t>none</t>
+  </si>
+  <si>
+    <t>SRMA00000000</t>
+  </si>
+  <si>
+    <t>GHNV00000000</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6084/m9.figshare.c.4437488</t>
+  </si>
+  <si>
     <t>10.1038/s41597-019-0254-8</t>
   </si>
   <si>
+    <t>https://doi.org/10.5061/dryad.119f80q</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.18112/openneuro.ds002179.v1.1.0</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2020.105653</t>
   </si>
   <si>
+    <t>no dataset to be downloaded</t>
+  </si>
+  <si>
     <t>10.1038/s41597-020-00597-w</t>
   </si>
   <si>
+    <t>https://doi.org/10.6084/m9.figshare.c.4869732</t>
+  </si>
+  <si>
+    <t>http://www.vocaltractlab.de/dvtd.zip</t>
+  </si>
+  <si>
     <t>10.1038/s41597-020-00773-y</t>
   </si>
   <si>
+    <t>https://zenodo.org/records/4059716</t>
+  </si>
+  <si>
     <t>10.1038/s41597-020-0487-6</t>
   </si>
   <si>
+    <t>https://www.ebi.ac.uk/pride/archive/projects/PXD016782</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.17632/nr7cs764rc.1</t>
+  </si>
+  <si>
     <t>10.1038/s41597-020-0495-6</t>
   </si>
   <si>
+    <t>https://physionet.org/content/ptb-xl/1.0.3/</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2021.107011</t>
   </si>
   <si>
+    <t>https://doi.org/10.17632/fzcmhhjs76.3</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2021.107320</t>
   </si>
   <si>
+    <t>GSE173610</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2021.107604</t>
   </si>
   <si>
+    <t>https://doi.org/10.17632/mtd59df24s.2</t>
+  </si>
+  <si>
     <t>10.1038/s41597-021-00913-y</t>
   </si>
   <si>
+    <t>https://doi.org/10.6084/m9.figshare.c.5222051</t>
+  </si>
+  <si>
+    <t>only v1 as yet</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2022.108347</t>
   </si>
   <si>
+    <t>https://doi.org/10.17632/wrhr5862cb.1</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2022.108399</t>
   </si>
   <si>
+    <t>https://doi.org/10.17605/OSF.IO/D34Y5</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2022.108542</t>
   </si>
   <si>
+    <t>https://github.com/emilywavery/Radiomics-data-sharing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AGPL-3.0 license </t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2022.108649</t>
   </si>
   <si>
+    <t>https://doi.org/10.17632/vfpxcbk5bx.4</t>
+  </si>
+  <si>
     <t>10.1016/j.dib.2022.108739</t>
   </si>
   <si>
+    <t>https://doi.org/10.5281/zenodo.6481140</t>
+  </si>
+  <si>
     <t>10.1038/s41597-022-01401-7</t>
   </si>
   <si>
+    <t>https://doi.org/10.3886/ICPSR36684.v4</t>
+  </si>
+  <si>
+    <t>bespoke data use agreement</t>
+  </si>
+  <si>
+    <t>https://github.com/npnl/ATLAS/</t>
+  </si>
+  <si>
     <t>10.1038/s41597-022-01532-x</t>
   </si>
   <si>
+    <t>https://doi.org/10.6019/CHEMBL4495565</t>
+  </si>
+  <si>
+    <t>undetermined</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6084/m9.figshare.19316219.v1</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6084/m9.figshare.19298807.v2</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6084/m9.figshare.19255067.v3</t>
+  </si>
+  <si>
     <t>10.1038/s41597-022-01669-9</t>
   </si>
   <si>
+    <t>https://napkon.de/</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5281/zenodo.6576176</t>
+  </si>
+  <si>
     <t>10.1038/s41597-022-01806-4</t>
   </si>
   <si>
+    <t>https://openneuro.org/datasets/ds001226</t>
+  </si>
+  <si>
+    <t>version not indicated in article</t>
+  </si>
+  <si>
+    <t>https://openneuro.org/datasets/ds002080</t>
+  </si>
+  <si>
     <t>10.1038/s41597-022-01822-4</t>
-  </si>
-  <si>
-    <t>Charité article DOI</t>
-  </si>
-  <si>
-    <t>data in repository (1 = yes, 0 = no)</t>
-  </si>
-  <si>
-    <t>dataset DOI, accession code, or link</t>
-  </si>
-  <si>
-    <t>dataset publication year (earliest version)</t>
-  </si>
-  <si>
-    <t>dataset publication year (version listed here)</t>
-  </si>
-  <si>
-    <t>license</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2016.02.047</t>
-  </si>
-  <si>
-    <t>NaN</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2016.06.021</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2016.07.009</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2016.09.012</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2017.08.034</t>
-  </si>
-  <si>
-    <t>10.1016/j.dib.2017.11.062</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.18112/openneuro.ds001875.v1.0.3</t>
-  </si>
-  <si>
-    <t>CC0</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.5281/zenodo.1471588</t>
-  </si>
-  <si>
-    <t>CC-BY</t>
-  </si>
-  <si>
-    <t>SRP136594</t>
-  </si>
-  <si>
-    <t>no versioning</t>
-  </si>
-  <si>
-    <t>none</t>
-  </si>
-  <si>
-    <t>SRMA00000000</t>
-  </si>
-  <si>
-    <t>GHNV00000000</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.c.4437488</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.5061/dryad.119f80q</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.18112/openneuro.ds002179.v1.1.0</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.c.4869732</t>
-  </si>
-  <si>
-    <t>http://www.vocaltractlab.de/dvtd.zip</t>
-  </si>
-  <si>
-    <t>https://zenodo.org/records/4059716</t>
-  </si>
-  <si>
-    <t>https://www.ebi.ac.uk/pride/archive/projects/PXD016782</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17632/nr7cs764rc.1</t>
-  </si>
-  <si>
-    <t>https://physionet.org/content/ptb-xl/1.0.3/</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17632/fzcmhhjs76.3</t>
-  </si>
-  <si>
-    <t>GSE173610</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17632/mtd59df24s.2</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.c.5222051</t>
-  </si>
-  <si>
-    <t>only v1 as yet</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17632/wrhr5862cb.1</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17605/OSF.IO/D34Y5</t>
-  </si>
-  <si>
-    <t>https://github.com/emilywavery/Radiomics-data-sharing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AGPL-3.0 license </t>
-  </si>
-  <si>
-    <t>https://doi.org/10.17632/vfpxcbk5bx.4</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.5281/zenodo.6481140</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.3886/ICPSR36684.v4</t>
-  </si>
-  <si>
-    <t>bespoke data use agreement</t>
-  </si>
-  <si>
-    <t>https://github.com/npnl/ATLAS/</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6019/CHEMBL4495565</t>
-  </si>
-  <si>
-    <t>undetermined</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.19316219.v1</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.19298807.v2</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.6084/m9.figshare.19255067.v3</t>
-  </si>
-  <si>
-    <t>https://napkon.de/</t>
-  </si>
-  <si>
-    <t>no dataset to be downloaded</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.5281/zenodo.6576176</t>
-  </si>
-  <si>
-    <t>https://openneuro.org/datasets/ds001226</t>
-  </si>
-  <si>
-    <t>version not indicated in article</t>
-  </si>
-  <si>
-    <t>https://openneuro.org/datasets/ds002080</t>
   </si>
   <si>
     <t>https://doi.org/10.17605/OSF.IO/8MBRU</t>
@@ -274,7 +285,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -859,7 +870,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1156,190 +1167,190 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B12FC64-94EA-495B-93DE-60284AA0C2A0}">
   <dimension ref="A1:H48"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="28.453125" customWidth="1"/>
-    <col min="3" max="3" width="6.54296875" customWidth="1"/>
-    <col min="4" max="4" width="66.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.1796875" customWidth="1"/>
-    <col min="6" max="6" width="53.1796875" customWidth="1"/>
-    <col min="7" max="7" width="21.81640625" customWidth="1"/>
-    <col min="8" max="8" width="33.453125" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="3" max="3" width="6.5703125" customWidth="1"/>
+    <col min="4" max="4" width="66.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.140625" customWidth="1"/>
+    <col min="6" max="6" width="53.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.85546875" customWidth="1"/>
+    <col min="8" max="8" width="33.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="14.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="14.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E2" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="14.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G3" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="14.45">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.45">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F5" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.45">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F6" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="14.45">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F7" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="20.25" customHeight="1">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E8" s="4">
         <v>2019</v>
@@ -1348,21 +1359,21 @@
         <v>2019</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="20.25" customHeight="1">
       <c r="A9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E9">
         <v>2019</v>
@@ -1371,90 +1382,90 @@
         <v>2019</v>
       </c>
       <c r="G9" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="26.25" customHeight="1">
       <c r="A10">
         <v>8</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C10" s="5">
         <v>1</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="E10" s="6">
         <v>2019</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="20.25" customHeight="1">
       <c r="A11">
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C11" s="5">
         <v>1</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>43</v>
+        <v>23</v>
       </c>
       <c r="E11" s="7">
         <v>2019</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="20.25" customHeight="1">
       <c r="A12">
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C12" s="5">
         <v>1</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="E12" s="6">
         <v>2019</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="20.25" customHeight="1">
       <c r="A13">
         <v>8</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C13" s="5">
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="E13">
         <v>2019</v>
@@ -1463,21 +1474,21 @@
         <v>2019</v>
       </c>
       <c r="G13" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="20.25" customHeight="1">
       <c r="A14">
         <v>9</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="C14" s="5">
         <v>1</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>46</v>
+        <v>27</v>
       </c>
       <c r="E14">
         <v>2019</v>
@@ -1486,21 +1497,21 @@
         <v>2019</v>
       </c>
       <c r="G14" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="20.25" customHeight="1">
       <c r="A15">
         <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="C15" s="5">
         <v>1</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>47</v>
+        <v>28</v>
       </c>
       <c r="E15">
         <v>2019</v>
@@ -1509,44 +1520,44 @@
         <v>2019</v>
       </c>
       <c r="G15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="20.25" customHeight="1">
       <c r="A16">
         <v>10</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="C16" s="5">
         <v>0</v>
       </c>
       <c r="D16" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" t="s">
         <v>30</v>
       </c>
-      <c r="E16" t="s">
-        <v>74</v>
-      </c>
       <c r="F16" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="20.25" customHeight="1">
       <c r="A17">
         <v>11</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C17" s="5">
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E17" s="5">
         <v>2020</v>
@@ -1555,44 +1566,44 @@
         <v>2020</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="20.25" customHeight="1">
       <c r="A18">
         <v>11</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C18" s="5">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="E18">
         <v>2020</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G18" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="20.25" customHeight="1">
       <c r="A19">
         <v>12</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="C19" s="5">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E19">
         <v>2020</v>
@@ -1601,44 +1612,44 @@
         <v>2020</v>
       </c>
       <c r="G19" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="21.75" customHeight="1">
       <c r="A20">
         <v>13</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C20" s="5">
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E20">
         <v>2020</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G20" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="20.25" customHeight="1">
       <c r="A21">
         <v>13</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C21" s="5">
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="E21" s="8">
         <v>2020</v>
@@ -1647,21 +1658,21 @@
         <v>2020</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="20.25" customHeight="1">
       <c r="A22">
         <v>14</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="C22">
         <v>1</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E22">
         <v>2020</v>
@@ -1670,21 +1681,21 @@
         <v>2022</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="20.25" customHeight="1">
       <c r="A23">
         <v>15</v>
       </c>
       <c r="B23" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C23">
         <v>1</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="E23">
         <v>2020</v>
@@ -1693,44 +1704,44 @@
         <v>2021</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="20.25" customHeight="1">
       <c r="A24">
         <v>16</v>
       </c>
       <c r="B24" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="C24">
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="E24">
         <v>2021</v>
       </c>
       <c r="F24" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G24" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="20.25" customHeight="1">
       <c r="A25">
         <v>17</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="C25">
         <v>1</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="E25">
         <v>2020</v>
@@ -1739,44 +1750,44 @@
         <v>2021</v>
       </c>
       <c r="G25" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="20.25" customHeight="1">
       <c r="A26">
         <v>18</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="C26">
         <v>1</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E26">
         <v>2021</v>
       </c>
       <c r="F26" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G26" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="20.25" customHeight="1">
       <c r="A27">
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
       <c r="C27">
         <v>1</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="E27">
         <v>2022</v>
@@ -1785,67 +1796,67 @@
         <v>2022</v>
       </c>
       <c r="G27" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="20.25" customHeight="1">
       <c r="A28">
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="C28">
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E28">
         <v>2021</v>
       </c>
       <c r="F28" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G28" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="20.25" customHeight="1">
       <c r="A29">
         <v>21</v>
       </c>
       <c r="B29" t="s">
-        <v>15</v>
+        <v>54</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="E29">
         <v>2022</v>
       </c>
       <c r="F29" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G29" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="20.25" customHeight="1">
       <c r="A30">
         <v>22</v>
       </c>
       <c r="B30" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="C30">
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="E30">
         <v>2022</v>
@@ -1854,44 +1865,44 @@
         <v>2022</v>
       </c>
       <c r="G30" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="20.25" customHeight="1">
       <c r="A31">
         <v>23</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="C31" s="5">
         <v>1</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E31">
         <v>2022</v>
       </c>
       <c r="F31" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G31" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="20.25" customHeight="1">
       <c r="A32">
         <v>24</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="C32" s="5">
         <v>1</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E32">
         <v>2017</v>
@@ -1900,222 +1911,222 @@
         <v>2021</v>
       </c>
       <c r="G32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="20.25" customHeight="1">
       <c r="A33">
         <v>24</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="C33" s="5">
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="E33">
         <v>2021</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G33" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="20.25" customHeight="1">
       <c r="A34">
         <v>25</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="C34" s="5">
         <v>1</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E34" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G34" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="20.25" customHeight="1">
       <c r="A35">
         <v>25</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="C35" s="5">
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E35">
         <v>2022</v>
       </c>
       <c r="F35" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G35" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="20.25" customHeight="1">
       <c r="A36">
         <v>25</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="C36" s="5">
         <v>1</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E36">
         <v>2022</v>
       </c>
       <c r="F36" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G36" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="20.25" customHeight="1">
       <c r="A37">
         <v>25</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="C37" s="5">
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E37">
         <v>2022</v>
       </c>
       <c r="F37" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G37" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="20.25" customHeight="1">
       <c r="A38">
         <v>26</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="C38" s="5">
         <v>1</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E38" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="F38" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G38" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="20.25" customHeight="1">
       <c r="A39">
         <v>26</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="C39" s="5">
         <v>1</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E39">
         <v>2022</v>
       </c>
       <c r="F39" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="G39" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="20.25" customHeight="1">
       <c r="A40">
         <v>27</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="C40" s="5">
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E40">
         <v>2018</v>
       </c>
       <c r="F40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G40" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="20.25" customHeight="1">
       <c r="A41">
         <v>27</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>21</v>
+        <v>74</v>
       </c>
       <c r="C41" s="5">
         <v>1</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E41">
         <v>2019</v>
       </c>
       <c r="F41" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G41" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="20.25" customHeight="1">
       <c r="A42">
         <v>28</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="C42" s="5">
         <v>1</v>
@@ -2127,18 +2138,18 @@
         <v>2017</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>41</v>
+        <v>21</v>
       </c>
       <c r="G42" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="20.25" customHeight="1">
       <c r="A43">
         <v>28</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="C43" s="5">
         <v>1</v>
@@ -2147,16 +2158,16 @@
         <v>80</v>
       </c>
       <c r="E43" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="F43" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G43" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="14.5" x14ac:dyDescent="0.35">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="14.45">
       <c r="H48" s="1"/>
     </row>
   </sheetData>
@@ -2199,19 +2210,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="11" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e8d63f71233e6ab4f1b448a0a865ebeb">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" xmlns:ns3="a0e84d40-090a-490d-8a02-2942ffba970a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bb36b253229a145d32e7027f701a87f0" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e9f9ff5d6d11740361dd8a7dc991dedf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" xmlns:ns3="a0e84d40-090a-490d-8a02-2942ffba970a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c17a16944702ffd78f9069df3a1f15a8" ns2:_="" ns3:_="">
     <xsd:import namespace="aaacefca-f467-416c-abd0-2b181dff1e20"/>
     <xsd:import namespace="a0e84d40-090a-490d-8a02-2942ffba970a"/>
     <xsd:element name="properties">
@@ -2265,7 +2274,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Bildmarkierungen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2375ea7b-1eef-4e91-915e-32e4cb5a9c34" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2375ea7b-1eef-4e91-915e-32e4cb5a9c34" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -2314,8 +2323,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Inhaltstyp"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titel"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -2405,33 +2414,24 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2D3F5D9-F66A-401E-BC58-4588B5177296}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a0e84d40-090a-490d-8a02-2942ffba970a"/>
-    <ds:schemaRef ds:uri="aaacefca-f467-416c-abd0-2b181dff1e20"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{647AA23E-A486-48B9-BA40-113933E28953}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53C58485-CAA4-48EF-8FCF-5133E95C879D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4AC41760-665F-4F7A-BEB6-2D76F0A5081C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{647AA23E-A486-48B9-BA40-113933E28953}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C2D3F5D9-F66A-401E-BC58-4588B5177296}"/>
 </file>
</xml_diff>